<commit_message>
Agora, o login funciona ✅
</commit_message>
<xml_diff>
--- a/excel_table.xlsx
+++ b/excel_table.xlsx
@@ -1,106 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="300" windowWidth="18735" windowHeight="11700"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Database do Banco</t>
-  </si>
-  <si>
-    <t>Nome</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>CPF</t>
-  </si>
-  <si>
-    <t>E-mail</t>
-  </si>
-  <si>
-    <t>Senha</t>
-  </si>
-  <si>
-    <t>Limite</t>
-  </si>
-  <si>
-    <t>Saldo</t>
-  </si>
-  <si>
-    <t>vinicius.generico@orkut.com</t>
-  </si>
-  <si>
-    <t>000000</t>
-  </si>
-  <si>
-    <t>Vinicius Anthony</t>
-  </si>
-  <si>
-    <t>Kalel Alessandro</t>
-  </si>
-  <si>
-    <t>kalel.emailaleatorio@gmail.com</t>
-  </si>
-  <si>
-    <t>Nicolas Mário</t>
-  </si>
-  <si>
-    <t>nicolas.supermario@yahoo.com</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="3">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -108,43 +45,101 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Escritório">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -182,7 +177,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Escritório">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -252,7 +247,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Escritório">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,135 +420,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cpf</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>password</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>cred_lim</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>bal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Vinicius Anthony</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>12668746448</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>vinicius.generico@orkut.com</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>123123</v>
+      </c>
+      <c r="F2" t="n">
+        <v>800</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kalel Alessandro</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>31025648548</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>kalel.emailaleatorio@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F3" t="n">
+        <v>120</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2400</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nicolas Mário</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>12668746448</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2">
-        <v>123123</v>
-      </c>
-      <c r="F3" s="4">
-        <v>800</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>31025648548</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="6">
-        <v>120</v>
-      </c>
-      <c r="G4" s="6">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
+      <c r="C4" t="n">
         <v>79215620110</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nicolas.supermario@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>69420</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F4" t="n">
         <v>1300</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G4" t="n">
         <v>700</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1"/>
-    <hyperlink ref="D4" r:id="rId2"/>
-    <hyperlink ref="D5" r:id="rId3"/>
-  </hyperlinks>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
-  <ignoredErrors>
-    <ignoredError sqref="E4" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sistema de criação de conta, mais funções e criação de config.py
</commit_message>
<xml_diff>
--- a/excel_table.xlsx
+++ b/excel_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>800</v>
       </c>
       <c r="G2" t="n">
-        <v>651</v>
+        <v>670</v>
       </c>
     </row>
     <row r="3">
@@ -544,6 +544,85 @@
       </c>
       <c r="G4" t="n">
         <v>700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Eduardo Gabriel</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>18064525122</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>edbiel@emailgenerico.com</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>789520</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sidney Rodrigues</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>41091448122</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>profsidneyrod@emailfalso.com</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>123456</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Marcos Eduardo</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15496525122</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>marc_eduardo@emailfalso.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>150670</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correção do sistema de login (que crashava caso a conta não fosse achada no login)
</commit_message>
<xml_diff>
--- a/excel_table.xlsx
+++ b/excel_table.xlsx
@@ -489,7 +489,7 @@
         <v>800</v>
       </c>
       <c r="G2" t="n">
-        <v>670</v>
+        <v>570</v>
       </c>
     </row>
     <row r="3">
@@ -605,20 +605,16 @@
       <c r="B7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>15496525122</t>
-        </is>
+      <c r="C7" t="n">
+        <v>15496525122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>marc_eduardo@emailfalso.com</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>150670</t>
-        </is>
+      <c r="E7" t="n">
+        <v>150670</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">

</xml_diff>

<commit_message>
Consertei o sistema de criação de conta (dnv😑)
</commit_message>
<xml_diff>
--- a/excel_table.xlsx
+++ b/excel_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -621,6 +621,60 @@
         <v>0</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vinicius Rocha</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>16958014220</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>rochassauro@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>150150</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carlos Eliezer</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>16351014015</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>carlinhosdograu@correspondencia.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>420420</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>